<commit_message>
Replaced fillpdf lib with own version
</commit_message>
<xml_diff>
--- a/test/test_cfg_pdf/rows.xlsx
+++ b/test/test_cfg_pdf/rows.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Martin\Documents\git_repos\school_report_tool\test\test_cfg_pdf_2_resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\git\kevin\test\test_cfg_pdf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CA32EC7-9F44-4560-97B3-9B30635B94F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{792A18D5-07EE-42C1-9901-2E112C41946F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2775" yWindow="555" windowWidth="15375" windowHeight="8820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8532" yWindow="4884" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Namen" sheetId="1" r:id="rId1"/>
@@ -278,7 +278,7 @@
     <t>__name</t>
   </si>
   <si>
-    <t>__0</t>
+    <t>__7</t>
   </si>
 </sst>
 </file>

</xml_diff>